<commit_message>
Elenca i valori ammessi nel modello, per chi lo apre con Numbers
Numbers non importa le tendine di Excel: i valori validi per Tipo e Stato
finiscono anche nel foglio Istruzioni, cosi' restano a portata di mano.
Il README spiega come passare da Numbers senza rompere il ciclo di
importazione.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Modello_inventario.xlsx
+++ b/docs/Modello_inventario.xlsx
@@ -737,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -853,26 +853,64 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Gli iPhone non si importano</t>
+          <t>Valori ammessi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sono gestiti solo a mano dal programma e non compaiono ne' nelle</t>
+          <t>Tipo:  Laptop,  Tablet</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>importazioni ne' nelle esportazioni. Se ne inserisci qui, vengono</t>
+          <t>Stato: Disponibile,  In attesa ritiro,  Guasto in attesa tecnico,  Da rebuildare,  Controllare</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
+        <is>
+          <t>Le tendine funzionano in Excel e in LibreOffice. Numbers non le</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>importa: in quel caso scrivi i valori qui sopra, sono gli stessi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Gli iPhone non si importano</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sono gestiti solo a mano dal programma e non compaiono ne' nelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>importazioni ne' nelle esportazioni. Se ne inserisci qui, vengono</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>ignorati.</t>
         </is>

</xml_diff>